<commit_message>
fixing cost price in new Item creation
</commit_message>
<xml_diff>
--- a/permissions list and description updated.xlsx
+++ b/permissions list and description updated.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="610" uniqueCount="513">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="608" uniqueCount="511">
   <si>
     <t>id</t>
   </si>
@@ -1544,12 +1544,6 @@
   </si>
   <si>
     <t>عرض وحدات القياس</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   costs.view </t>
-  </si>
-  <si>
-    <t xml:space="preserve">   finance.view </t>
   </si>
   <si>
     <t xml:space="preserve">   inventory_adjustment.view </t>
@@ -1568,8 +1562,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1624,9 +1626,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1635,6 +1637,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1937,7 +1940,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E101"/>
+  <dimension ref="A1:E103"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="4.6328125" bestFit="1" customWidth="1"/>
@@ -3561,34 +3564,30 @@
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="B96" t="s">
-        <v>507</v>
+      <c r="B96" s="4" t="s">
+        <v>509</v>
       </c>
     </row>
     <row r="97" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B97" t="s">
-        <v>508</v>
+      <c r="B97" s="4" t="s">
+        <v>510</v>
       </c>
     </row>
     <row r="98" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B98" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
     </row>
     <row r="99" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B99" t="s">
-        <v>510</v>
-      </c>
-    </row>
-    <row r="100" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B100" t="s">
-        <v>511</v>
-      </c>
-    </row>
-    <row r="101" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B101" t="s">
-        <v>512</v>
-      </c>
+        <v>508</v>
+      </c>
+    </row>
+    <row r="102" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B102" s="4"/>
+    </row>
+    <row r="103" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B103" s="4"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:E95">
@@ -3597,6 +3596,7 @@
     </sortState>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>